<commit_message>
SPM-81 Rebuild test case workbook with each case's summary on its sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-81_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-81_Test_Cases.xlsx
@@ -1137,7 +1137,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -1164,13 +1164,25 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="98.5" customHeight="1">
+    <row r="3" ht="31" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>An event with a single venue booking is shown as before: one room on the Overview and one request on the Venue tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="98.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>`npm run fixtures:spm81` has been run since the last full `npx prisma db seed`.
 'SPM81 Solo Workshop' has one Approved booking, at SPM81 Auditorium on 26 Aug 2027, 09:00–12:00.
@@ -1179,88 +1191,80 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="44.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+    <row r="5" ht="44.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>1. Click 'All Events' in the sidebar and open 'SPM81 Solo Workshop'
 2. Click the 'Venue' tab</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="31" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+    <row r="6" ht="31" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Event: SPM81 Solo Workshop | When: 26 Aug 2027, 09:00–12:00
 Booking: SPM81 Auditorium (SPM81-AUD), Approved, 09:00–12:00</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="98.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+    <row r="7" ht="98.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Step 1: On the Overview, the 'Venue' row reads 'SPM81 Auditorium (SPM81-AUD)' and nothing else.
 Step 2: The 'Booking requests' card lists one request: 'SPM81 Auditorium (SPM81-AUD)' with '26 Aug 2027, 09:00–12:00 · Theatre' and the 'Approved' badge. The venue list below it is unchanged: each suitable venue has 'Suitable' and a 'Request booking' button.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>kayalvizhi24</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B9" s="14" t="n">
         <v>46305</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
+          <t>Actual Result</t>
         </is>
       </c>
       <c r="B12" s="3" t="n"/>
@@ -1268,7 +1272,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>
@@ -1276,7 +1280,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Executed by</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B14" s="3" t="n"/>
@@ -1284,10 +1288,18 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1300,7 +1312,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -1327,13 +1339,25 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="98.5" customHeight="1">
+    <row r="3" ht="44.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>A second session of the same event cannot request a room one of its sessions already holds at overlapping times, but can take it as that session ends</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="98.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Run `npm run fixtures:spm81` before this case, and again after it: the case sends one booking request.
 'SPM81 Parallel Tracks' has three sessions on 24 Aug 2027. Its 'Morning plenary' session has a Pending request at SPM81 Auditorium for 09:00–12:00.
@@ -1341,13 +1365,13 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="179.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+    <row r="5" ht="179.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>1. Click 'All Events' in the sidebar and open 'SPM81 Parallel Tracks'
 2. Click the 'Venue' tab
@@ -1362,13 +1386,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="112" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+    <row r="6" ht="112" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Event: SPM81 Parallel Tracks | Sessions on 24 Aug 2027: 'Morning plenary' 09:00–12:00; 'Workshop' 10:00–12:00; 'Afternoon plenary' 12:00–15:00
 Existing: SPM81 Auditorium, Pending, for 'Morning plenary', 09:00–12:00
@@ -1376,13 +1400,13 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="220" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+    <row r="7" ht="220" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Step 2: The 'Booking requests' card lists 'SPM81 Auditorium (SPM81-AUD)' with 'Morning plenary · 24 Aug 2027, 09:00–12:00 · Theatre' and the 'Pending' badge.
 Step 5: The request is not sent. A red alert reads 'This event already has a pending request for SPM81 Auditorium on 24 Aug 2027, 09:00–12:00.'
@@ -1392,49 +1416,41 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>kayalvizhi24</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B9" s="14" t="n">
         <v>46305</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
+          <t>Actual Result</t>
         </is>
       </c>
       <c r="B12" s="3" t="n"/>
@@ -1442,7 +1458,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>
@@ -1450,7 +1466,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Executed by</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B14" s="3" t="n"/>
@@ -1458,10 +1474,18 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1474,7 +1498,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -1501,13 +1525,25 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="98.5" customHeight="1">
+    <row r="3" ht="31" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>After Venue Staff reject one venue, the same venue can be requested again, and the event's other booking is unchanged</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="98.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Run `npm run fixtures:spm81` before this case, and again after it: the case sends one booking request.
 'SPM81 Second Attempt' (31 Aug 2027, 09:00–12:00) has a Rejected request at SPM81 Auditorium and an Approved booking at SPM81 Breakout Room A.
@@ -1515,13 +1551,13 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="85" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+    <row r="5" ht="85" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>1. Click 'All Events' in the sidebar and open 'SPM81 Second Attempt'
 2. Click the 'Venue' tab
@@ -1531,13 +1567,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="71.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+    <row r="6" ht="71.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Event: SPM81 Second Attempt | When: 31 Aug 2027, 09:00–12:00
 Existing: SPM81 Auditorium, Rejected, reason 'Stage lighting is being serviced that morning.'; SPM81 Breakout Room A, Approved
@@ -1545,13 +1581,13 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="179.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+    <row r="7" ht="179.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Step 2: The 'Booking requests' card lists 'SPM81 Auditorium (SPM81-AUD)' with the 'Rejected' badge and 'Reason from Venue Staff: Stage lighting is being serviced that morning.', and 'SPM81 Breakout Room A (SPM81-BRA)' with the 'Approved' badge.
 Step 4: A green alert 'Booking request sent to Venue Staff.' is shown: a rejected request holds nothing, so asking for the same venue and times again is not a repeat.
@@ -1559,49 +1595,41 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>kayalvizhi24</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B9" s="14" t="n">
         <v>46305</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
+          <t>Actual Result</t>
         </is>
       </c>
       <c r="B12" s="3" t="n"/>
@@ -1609,7 +1637,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>
@@ -1617,7 +1645,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Executed by</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B14" s="3" t="n"/>
@@ -1625,10 +1653,18 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1641,7 +1677,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -1668,13 +1704,25 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="85" customHeight="1">
+    <row r="3" ht="44.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Venue Staff can approve two venues for the same event at the same times; the second approval is not treated as a conflict</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="85" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Run `npm run fixtures:spm81` before this case, and again after it: the case approves two booking requests.
 'SPM81 Twin Rooms' has two Pending requests for 2 Sep 2027, 09:00–12:00: one at SPM81 Auditorium and one at SPM81 Breakout Room A.
@@ -1682,13 +1730,13 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="179.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+    <row r="5" ht="179.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>1. Log in as marcus.wong@connectsphere.com / password123
 2. Click 'Booking Requests' in the sidebar
@@ -1703,26 +1751,26 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="44.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+    <row r="6" ht="44.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Event: SPM81 Twin Rooms | When: 2 Sep 2027, 09:00–12:00
 Requests: SPM81 Auditorium (SPM81-AUD), Pending; SPM81 Breakout Room A (SPM81-BRA), Pending</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="206.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+    <row r="7" ht="206.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Step 4: A green alert 'Booking approved' reads 'SPM81 Auditorium (SPM81-AUD) for &lt;reference&gt; SPM81 Twin Rooms on 2 Sep 2027, 09:00–12:00 is now Approved — the room is booked.'
 Step 5: The 'SPM81 Breakout Room A' card has no 'Conflict' badge and its 'Approve' button is enabled, although the same event now holds the Auditorium for the same times. The 'Approve this booking?' dialog opens.
@@ -1732,49 +1780,41 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>kayalvizhi24</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B9" s="14" t="n">
         <v>46305</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
+          <t>Actual Result</t>
         </is>
       </c>
       <c r="B12" s="3" t="n"/>
@@ -1782,7 +1822,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>
@@ -1790,7 +1830,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Executed by</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B14" s="3" t="n"/>
@@ -1798,10 +1838,18 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1916,7 +1964,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -1943,26 +1991,38 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="44.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>The Coordinator requests two different venues for the same event at the same date and times, and both requests are accepted and listed together</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="71.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Run `npm run fixtures:spm81` from the project folder before this case (it only touches the 'SPM81 …' events and venues, never anyone else's data). Run it again after this case: the case sends two booking requests.
 Logged out.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="152.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+    <row r="5" ht="152.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>1. Log in as daniel.tan@connectsphere.com / password123
 2. Click 'All Events' in the sidebar and open 'SPM81 Leadership Summit'
@@ -1976,13 +2036,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="98.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+    <row r="6" ht="98.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Event: SPM81 Leadership Summit | When: 3 Aug 2027, 09:00–17:00 | No sessions | Status: Planning | No booking requests yet
 Venues: SPM81 Auditorium (SPM81-AUD), setup 30 min, turnaround 30 min; SPM81 Breakout Room A (SPM81-BRA), no setup or turnaround
@@ -1990,13 +2050,13 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="260.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+    <row r="7" ht="260.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Step 4: The 'Request a venue booking' page opens for 'SPM81 Leadership Summit' at 'SPM81 Auditorium (SPM81-AUD)'. 'Date' shows 3 Aug 2027, 'Start time' 09:00 and 'End time' 17:00, with 'Room in use: 08:30–17:30'.
 Step 5: A green alert 'Booking request sent to Venue Staff.' is shown.
@@ -2007,49 +2067,41 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>kayalvizhi24</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B9" s="14" t="n">
         <v>46305</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
+          <t>Actual Result</t>
         </is>
       </c>
       <c r="B12" s="3" t="n"/>
@@ -2057,7 +2109,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>
@@ -2065,7 +2117,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Executed by</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B14" s="3" t="n"/>
@@ -2073,10 +2125,18 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2089,7 +2149,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -2116,26 +2176,38 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="58" customHeight="1">
+    <row r="3" ht="44.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>For a multi-session event, two venues can be requested for the same session, and each request is listed with that session</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Run `npm run fixtures:spm81` before this case, and again after it: the case sends two booking requests.
 Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123), the coordinator assigned to every 'SPM81 …' event.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="179.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+    <row r="5" ht="179.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>1. Click 'All Events' in the sidebar and open 'SPM81 Two-Track Conference'
 2. Click the 'Venue' tab
@@ -2149,26 +2221,26 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Event: SPM81 Two-Track Conference | Sessions: 'Day 1' 5 Aug 2027, 09:00–12:00; 'Day 2' 6 Aug 2027, 09:00–12:00
 Both venues requested for the Day 1 session, 5 Aug 2027, 09:00–12:00</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="179.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+    <row r="7" ht="179.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Step 4: The 'Request a venue booking' page shows 'Session: Day 1 — 5 Aug 2027, 09:00–12:00' and 'Venue: SPM81 Auditorium (SPM81-AUD)'.
 Step 5: A green alert 'Booking request sent to Venue Staff.' is shown.
@@ -2178,49 +2250,41 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>kayalvizhi24</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B9" s="14" t="n">
         <v>46305</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
+          <t>Actual Result</t>
         </is>
       </c>
       <c r="B12" s="3" t="n"/>
@@ -2228,7 +2292,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>
@@ -2236,7 +2300,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Executed by</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B14" s="3" t="n"/>
@@ -2244,10 +2308,18 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2260,7 +2332,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -2287,13 +2359,25 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="125.5" customHeight="1">
+    <row r="3" ht="44.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>A venue that is unavailable, and one that is already booked by another event, are each refused on their own, and a third venue can still be requested for the same times</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="125.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Run `npm run fixtures:spm81` before this case, and again after it: the case sends one booking request.
 'SPM81 Rival Booking' holds an Approved booking at SPM81 Auditorium on 10 Aug 2027, 10:00–12:00 (room in use 09:30–12:30).
@@ -2302,13 +2386,13 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="193" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+    <row r="5" ht="193" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>1. Click 'All Events' in the sidebar and open 'SPM81 Sales Kickoff'
 2. Click the 'Venue' tab
@@ -2324,13 +2408,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="98.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+    <row r="6" ht="98.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Event: SPM81 Sales Kickoff | When: 10 Aug 2027, 10:00–12:00 | No booking requests yet
 SPM81 Breakout Room B: unavailable 10 Aug 2027, 08:00–13:00 (maintenance)
@@ -2339,13 +2423,13 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="206.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+    <row r="7" ht="206.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Step 4: The request is not sent. A red alert reads 'SPM81 Breakout Room B is unavailable at this time (maintenance, 10 Aug 2027, 08:00–13:00).'
 Step 5: The Venue tab opens and no booking request has been added. 'Request booking' is still offered on the other two venues.
@@ -2355,49 +2439,41 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>kayalvizhi24</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B9" s="14" t="n">
         <v>46305</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
+          <t>Actual Result</t>
         </is>
       </c>
       <c r="B12" s="3" t="n"/>
@@ -2405,7 +2481,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>
@@ -2413,7 +2489,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Executed by</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B14" s="3" t="n"/>
@@ -2421,10 +2497,18 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2437,7 +2521,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -2464,13 +2548,25 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="112" customHeight="1">
+    <row r="3" ht="31" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>A venue the event has already requested or booked cannot be requested again for the same or overlapping times</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="112" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>`npm run fixtures:spm81` has been run since the last full `npx prisma db seed`.
 'SPM81 Repeat Request' has a Pending request at SPM81 Auditorium and an Approved booking at SPM81 Breakout Room A, both for 12 Aug 2027, 09:00–12:00.
@@ -2479,13 +2575,13 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="166" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+    <row r="5" ht="166" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>1. Click 'All Events' in the sidebar and open 'SPM81 Repeat Request'
 2. Click the 'Venue' tab
@@ -2499,13 +2595,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="71.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+    <row r="6" ht="71.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Event: SPM81 Repeat Request | When: 12 Aug 2027, 09:00–12:00
 Existing: SPM81 Auditorium, Pending, 09:00–12:00; SPM81 Breakout Room A, Approved, 09:00–12:00
@@ -2513,13 +2609,13 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="220" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+    <row r="7" ht="220" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Step 2: The 'Booking requests' card lists 'SPM81 Auditorium (SPM81-AUD)' with the 'Pending' badge and 'SPM81 Breakout Room A (SPM81-BRA)' with the 'Approved' badge, each with '12 Aug 2027, 09:00–12:00 · Theatre'.
 Step 4: The request is not sent. A red alert reads 'This event already has a pending request for SPM81 Auditorium on 12 Aug 2027, 09:00–12:00.'
@@ -2529,49 +2625,41 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>kayalvizhi24</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B9" s="14" t="n">
         <v>46305</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
+          <t>Actual Result</t>
         </is>
       </c>
       <c r="B12" s="3" t="n"/>
@@ -2579,7 +2667,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>
@@ -2587,7 +2675,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Executed by</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B14" s="3" t="n"/>
@@ -2595,10 +2683,18 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2611,7 +2707,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -2638,13 +2734,25 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="98.5" customHeight="1">
+    <row r="3" ht="31" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Venue Staff see each of an event's venue requests as its own card, and approving one leaves the other Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="98.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Run `npm run fixtures:spm81` before this case. Do not run it again afterwards: go straight on to SPM-81-TC06, and reset after that one.
 'SPM81 Partner Day' has two Pending requests for 17 Aug 2027, 09:00–12:00: one at SPM81 Auditorium and one at SPM81 Breakout Room A.
@@ -2652,13 +2760,13 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="71.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+    <row r="5" ht="71.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>1. Log in as marcus.wong@connectsphere.com / password123
 2. Click 'Booking Requests' in the sidebar
@@ -2667,26 +2775,26 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="44.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+    <row r="6" ht="44.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Event: SPM81 Partner Day | When: 17 Aug 2027, 09:00–12:00
 Requests: SPM81 Auditorium (SPM81-AUD), Pending; SPM81 Breakout Room A (SPM81-BRA), Pending</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="220" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+    <row r="7" ht="220" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Step 2: The 'Booking Requests' page lists two separate cards for 'SPM81 Partner Day': 'SPM81 Auditorium (SPM81-AUD)' and 'SPM81 Breakout Room A (SPM81-BRA)'. Each has its own 'Pending' badge, a 'Requested' row reading '17 Aug 2027, 09:00–12:00', and its own 'Approve' and 'Reject with a reason' buttons.
 Step 3: The 'Approve this booking?' dialog names only the Auditorium: 'This books SPM81 Auditorium (SPM81-AUD) for &lt;reference&gt; SPM81 Partner Day on 17 Aug 2027, 09:00–12:00.'
@@ -2694,49 +2802,41 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>kayalvizhi24</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B9" s="14" t="n">
         <v>46305</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
+          <t>Actual Result</t>
         </is>
       </c>
       <c r="B12" s="3" t="n"/>
@@ -2744,7 +2844,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>
@@ -2752,7 +2852,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Executed by</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B14" s="3" t="n"/>
@@ -2760,10 +2860,18 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2776,7 +2884,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -2803,13 +2911,25 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="85" customHeight="1">
+    <row r="3" ht="31" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Rejecting one of an event's venue requests leaves its other, approved booking unchanged</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="85" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>SPM-81-TC05 has just been run (SPM81 Auditorium is Approved for 'SPM81 Partner Day'; its request for SPM81 Breakout Room A is still Pending).
 Still logged in as Marcus Wong, on the 'Booking Requests' page.
@@ -2817,13 +2937,13 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="125.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+    <row r="5" ht="125.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>1. Find the 'SPM81 Breakout Room A' card for 'SPM81 Partner Day' (use Ctrl+F) and click 'Reject with a reason'
 2. Type the reason in 'Reason for rejection' and click 'Reject request'
@@ -2834,25 +2954,25 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="31" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+    <row r="6" ht="31" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Reason for rejection: Breakout Room A is reserved for staff training that morning.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="179.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+    <row r="7" ht="179.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Step 2: A green alert 'Booking request rejected' reads 'SPM81 Breakout Room A (SPM81-BRA) for &lt;reference&gt; SPM81 Partner Day on 17 Aug 2027, 09:00–12:00 is now Rejected. The Coordinator can see your reason on the event's Venue tab.' The card leaves the list.
 Step 5: On the Overview, the 'Venue' row still reads 'SPM81 Auditorium (SPM81-AUD)'.
@@ -2860,49 +2980,41 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>kayalvizhi24</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B9" s="14" t="n">
         <v>46305</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
+          <t>Actual Result</t>
         </is>
       </c>
       <c r="B12" s="3" t="n"/>
@@ -2910,7 +3022,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>
@@ -2918,7 +3030,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Executed by</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B14" s="3" t="n"/>
@@ -2926,10 +3038,18 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2942,7 +3062,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.77734375" customWidth="1" min="1" max="1"/>
@@ -2969,13 +3089,25 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="112" customHeight="1">
+    <row r="3" ht="44.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>An event's venue bookings are shown together, each with its own venue, times and status, and the Overview names every approved room</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="112" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>`npm run fixtures:spm81` has been run since the last full `npx prisma db seed`.
 'SPM81 Showcase Day' (19 Aug 2027, 09:00–17:00) has three venue bookings: SPM81 Auditorium, Approved, 09:00–17:00; SPM81 Breakout Room A, Approved, 08:30–17:30; SPM81 Breakout Room B, Pending, 09:00–17:00.
@@ -2984,13 +3116,13 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="112" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+    <row r="5" ht="112" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>1. Log in as daniel.tan@connectsphere.com / password123
 2. Click 'All Events' in the sidebar and open 'SPM81 Showcase Day'
@@ -3001,13 +3133,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="71.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+    <row r="6" ht="71.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Event: SPM81 Showcase Day | When: 19 Aug 2027, 09:00–17:00
 Bookings: SPM81 Auditorium (SPM81-AUD), Approved, 09:00–17:00 | SPM81 Breakout Room A (SPM81-BRA), Approved, 08:30–17:30 | SPM81 Breakout Room B (SPM81-BRB), Pending, 09:00–17:00
@@ -3015,13 +3147,13 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="179.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+    <row r="7" ht="179.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Step 2: On the Overview, the 'Venue' row reads 'SPM81 Breakout Room A (SPM81-BRA) · SPM81 Auditorium (SPM81-AUD)': both approved rooms, and not SPM81 Breakout Room B, whose request is still Pending.
 Step 3: One 'Booking requests' card lists all three: 'SPM81 Auditorium (SPM81-AUD)' with '19 Aug 2027, 09:00–17:00 · Theatre' and 'Approved'; 'SPM81 Breakout Room A (SPM81-BRA)' with '19 Aug 2027, 08:30–17:30 · Theatre' and 'Approved'; 'SPM81 Breakout Room B (SPM81-BRB)' with '19 Aug 2027, 09:00–17:00 · Theatre' and 'Pending'.
@@ -3029,49 +3161,41 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>kayalvizhi24</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B9" s="14" t="n">
         <v>46305</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
+          <t>Actual Result</t>
         </is>
       </c>
       <c r="B12" s="3" t="n"/>
@@ -3079,7 +3203,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>
@@ -3087,7 +3211,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Executed by</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B14" s="3" t="n"/>
@@ -3095,10 +3219,18 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
SPM-81 Record the manual test pass and two known gaps
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-81_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-81_Test_Cases.xlsx
@@ -1887,13 +1887,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="98.5" customHeight="1">
+    <row r="2" ht="112" customHeight="1">
       <c r="A2" s="11" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Written 2026-10-10, before any SPM-81 code. Checked against Week 7 Customer Changes (Change #3), the discussion logs up to 20261006 (#41, #109, #128) and the code on main. Finding: the request rules already checked one venue at a time and exempted the event's own bookings (SPM-42, SPM-44, SPM-93), so nothing stopped a second venue. The only code SPM-81 changed is the AC4 rule below (built 2026-10-10, after the cases). None of the cases has been run by hand yet.</t>
+          <t>Written 2026-10-10, before any SPM-81 code. Checked against Week 7 Customer Changes (Change #3), the discussion logs up to 20261006 (#41, #109, #128) and the code on main. Finding: the request rules already checked one venue at a time and exempted the event's own bookings (SPM-42, SPM-44, SPM-93), so nothing stopped a second venue. The only code SPM-81 changed is the AC4 rule below (built 2026-10-10, after the cases). All 11 cases passed when run by hand on 2026-10-11 (kayalvizhi24), on the build with main merged in.</t>
         </is>
       </c>
       <c r="C2" s="11" t="n"/>

</xml_diff>